<commit_message>
fix(finance): master tracker reads PARTNER-SHEET-IDS.json
build_master_sheet.py had a hardcoded 10-partner SHEETS list, so uber,
rapido, ola, and noon never appeared despite registry + refresh uploads
targeting the same _master_tracker sheet. Derive rows from
PARTNER-SHEET-IDS.json with stable display order and notes.
</commit_message>
<xml_diff>
--- a/finance/_master-unit-econ.xlsx
+++ b/finance/_master-unit-econ.xlsx
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -671,140 +671,140 @@
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Saudi / Red Sea (PIF)</t>
+          <t>Bolt</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1K75Ln5YKgKkOBKnprAoVGu4KeuO83Dx2TGzQ-1o45Ig/edit","open ↗")</f>
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1XkD0x-PfDyY34ZBy5jX2u1LqoibAd_xMiyO-Re2UWUk/edit","open ↗")</f>
         <v/>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>0 / 1</t>
+          <t>63 / 139</t>
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0</v>
+        <v>527</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0</v>
+        <v>105876268</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>6</v>
+        <v>280</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>0</v>
+        <v>58220204</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>6</v>
+        <v>807</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>0</v>
+        <v>164096472</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Low-confidence / largely 2030-dated. Greenfield OFF. Treat as forward.</t>
+          <t>MENA grounded floor + Med/Baltic aspirational tail (Bucket C bound).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Red Sea Global</t>
+          <t>Yango</t>
         </is>
       </c>
       <c r="B7" s="10">
-        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1QbF7zSl-5CllYXXLRJvvKJXXBpOu8Cnl97X1rO5J77c/edit","open ↗")</f>
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1fvB_tc8IWUTlKMWjPcoJde_uPnGKVqoCxxsgd5IL1rM/edit","open ↗")</f>
         <v/>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>3 / 2</t>
+          <t>41 / 124</t>
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>235</v>
+        <v>284</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>162388864</v>
+        <v>79853143</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>12</v>
+        <v>227</v>
       </c>
       <c r="G7" s="12" t="n">
         <v>2387088</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>247</v>
+        <v>511</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>164775952</v>
+        <v>82240231</v>
       </c>
       <c r="J7" s="13" t="inlineStr">
         <is>
-          <t>Resort-operator corridors. Small, grounded subset.</t>
+          <t>MENA + Africa grounded + CIS/Caspian/Africa aspirational tail (Bucket C bound).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>JIH Global (Maldives)</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="B8" s="5">
-        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/136mve2Z-c2FRZm2cZZ3of9jk85kpEkpzf-ZIC9dzXJU/edit","open ↗")</f>
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/19VtRN0U6Gggq_RQlRuSxmiIxnp2KgGEIvXOW72RQHIQ/edit","open ↗")</f>
         <v/>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>38 / 5</t>
+          <t>63 / 87</t>
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>74</v>
+        <v>314</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>81100880</v>
+        <v>62292849</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>0</v>
+        <v>2927731</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>74</v>
+        <v>492</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>81100880</v>
+        <v>65220580</v>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Maldives 43 corridors geometry-bound; network-sum captive fleet.</t>
+          <t>Global mobility rollup; MENA + Med + Hawaii + LatAm scoped markets.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Rapido (India)</t>
         </is>
       </c>
       <c r="B9" s="10">
-        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1v0Fo-QDKVIEiMzzYUbrugCUH1cBJdLKD9URG1R16S0Q/edit","open ↗")</f>
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1ujRCwCKNFcfUbVL5B312fjcYmtvsDVhBtK2hsTHo-qA/edit","open ↗")</f>
         <v/>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>1 / 7</t>
+          <t>93 / 0</t>
         </is>
       </c>
       <c r="D9" s="11" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>2005817</v>
+        <v>1438983</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>0</v>
@@ -813,182 +813,338 @@
         <v>0</v>
       </c>
       <c r="H9" s="11" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>2005817</v>
+        <v>1438983</v>
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>Doha 4/4 in-range corridors bound. Banana Island captive carries floor.</t>
+          <t>PR #58 India — Mumbai/Goa/Kerala/Andaman sealed spine; ridehail archetype.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Bolt</t>
+          <t>Ola (India)</t>
         </is>
       </c>
       <c r="B10" s="5">
-        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1XkD0x-PfDyY34ZBy5jX2u1LqoibAd_xMiyO-Re2UWUk/edit","open ↗")</f>
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1pNwq_GQd2Fdem8O4o2GNNoKxBPxXOPDh1qfbhGFGkaQ/edit","open ↗")</f>
         <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>63 / 139</t>
+          <t>93 / 0</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>527</v>
+        <v>15</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>105876268</v>
+        <v>1438983</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>280</v>
+        <v>0</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>58220204</v>
+        <v>0</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>807</v>
+        <v>15</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>164096472</v>
+        <v>1438983</v>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>MENA grounded floor + Med/Baltic aspirational tail (Bucket C bound).</t>
+          <t>PR #58 India — same sealed spine as Rapido; ridehail archetype.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Yango</t>
+          <t>Noon (UAE)</t>
         </is>
       </c>
       <c r="B11" s="10">
-        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1fvB_tc8IWUTlKMWjPcoJde_uPnGKVqoCxxsgd5IL1rM/edit","open ↗")</f>
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1v0ywhNFk_fA1JRVhizWlz89RKgQWlID9RD3LfBhVB2Y/edit","open ↗")</f>
         <v/>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>41 / 124</t>
+          <t>8 / 0</t>
         </is>
       </c>
       <c r="D11" s="11" t="n">
-        <v>284</v>
+        <v>7</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>79853143</v>
+        <v>1343999</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>227</v>
+        <v>0</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>2387088</v>
+        <v>0</v>
       </c>
       <c r="H11" s="11" t="n">
-        <v>511</v>
+        <v>7</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>82240231</v>
+        <v>1343999</v>
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>MENA + Africa grounded + CIS/Caspian/Africa aspirational tail (Bucket C bound).</t>
+          <t>PR #58 UAE — 12 sealed super_app corridors; Careem-style demand ladder.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Constance (Maldives)</t>
+          <t>JIH Global (Maldives)</t>
         </is>
       </c>
       <c r="B12" s="5">
-        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1Lhz_6nh3HnCK8L7tzr4HhmNEtfnXx2smecYPNQSORl0/edit","open ↗")</f>
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/136mve2Z-c2FRZm2cZZ3of9jk85kpEkpzf-ZIC9dzXJU/edit","open ↗")</f>
         <v/>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>— / —</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="7" t="n"/>
+          <t>38 / 5</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>81100880</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>81100880</v>
+      </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>Captive resort-transfer; network-sum captive fleet. Greenfield OFF. [no agg-constance.json in finance/recal]</t>
+          <t>Maldives 43 corridors geometry-bound; network-sum captive fleet.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="B13" s="10">
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1v0Fo-QDKVIEiMzzYUbrugCUH1cBJdLKD9URG1R16S0Q/edit","open ↗")</f>
+        <v/>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>1 / 7</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>2005817</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>2005817</v>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>Doha 4/4 in-range corridors bound. Banana Island captive carries floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Saudi / Red Sea (PIF)</t>
+        </is>
+      </c>
+      <c r="B14" s="5">
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1K75Ln5YKgKkOBKnprAoVGu4KeuO83Dx2TGzQ-1o45Ig/edit","open ↗")</f>
+        <v/>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>0 / 1</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Low-confidence / largely 2030-dated. Greenfield OFF. Treat as forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Red Sea Global</t>
+        </is>
+      </c>
+      <c r="B15" s="10">
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1QbF7zSl-5CllYXXLRJvvKJXXBpOu8Cnl97X1rO5J77c/edit","open ↗")</f>
+        <v/>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>3 / 2</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>235</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>162388864</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>2387088</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>247</v>
+      </c>
+      <c r="I15" s="12" t="n">
+        <v>164775952</v>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>Resort-operator corridors. Small, grounded subset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Constance (Maldives)</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1Lhz_6nh3HnCK8L7tzr4HhmNEtfnXx2smecYPNQSORl0/edit","open ↗")</f>
+        <v/>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>— / —</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Captive resort-transfer; network-sum captive fleet. Greenfield OFF. [no agg-constance.json in /Users/jaideep/navier-atlas/finance/recal]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
           <t>Four Seasons (Maldives)</t>
         </is>
       </c>
-      <c r="B13" s="10">
+      <c r="B17" s="10">
         <f>HYPERLINK("https://docs.google.com/spreadsheets/d/1Flk6PfRgCNdSGlP49lf1KxXaoR4qdlLcs1O8YA72gcc/edit","open ↗")</f>
         <v/>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>— / —</t>
         </is>
       </c>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="12" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="12" t="n"/>
-      <c r="J13" s="13" t="inlineStr">
-        <is>
-          <t>Captive resort-transfer; network-sum captive fleet. Greenfield OFF. [no agg-four-seasons.json in finance/recal]</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="11" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>Captive resort-transfer; network-sum captive fleet. Greenfield OFF. [no agg-four-seasons.json in /Users/jaideep/navier-atlas/finance/recal]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>PORTFOLIO (gross)</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr"/>
-      <c r="C14" s="15" t="inlineStr"/>
-      <c r="D14" s="16">
-        <f>SUM(D4:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="17">
-        <f>SUM(E4:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="16">
-        <f>SUM(F4:F13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="17">
-        <f>SUM(G4:G13)</f>
-        <v/>
-      </c>
-      <c r="H14" s="16">
-        <f>SUM(H4:H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="17">
-        <f>SUM(I4:I13)</f>
-        <v/>
-      </c>
-      <c r="J14" s="18" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr"/>
+      <c r="C18" s="15" t="inlineStr"/>
+      <c r="D18" s="16">
+        <f>SUM(D4:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="17">
+        <f>SUM(E4:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="16">
+        <f>SUM(F4:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="17">
+        <f>SUM(G4:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="16">
+        <f>SUM(H4:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="17">
+        <f>SUM(I4:I17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
         <is>
           <t>Gross sum across partner scopes; not de-duplicated.</t>
         </is>

</xml_diff>